<commit_message>
chore: consolidate repository cleanup and adaptive OCR updates
</commit_message>
<xml_diff>
--- a/data/master/msds_index_V24.xlsx
+++ b/data/master/msds_index_V24.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="현재_통합_문서"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\안티그래비티\MSDS_Extraction_GPT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\안티그래비티\MSDS_Extraction_GPT\data\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C97DE4-C13B-4282-AA46-24AA6CB6D294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154EF211-B214-4818-B9EC-5EFD15E15598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="30960" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6709" uniqueCount="1592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6709" uniqueCount="1593">
   <si>
     <t>정렬코드</t>
   </si>
@@ -4816,6 +4816,10 @@
   </si>
   <si>
     <t>14807-96-6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7440-22-4</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -10744,7 +10748,7 @@
         <v>309</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>303</v>
+        <v>1592</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>100</v>

</xml_diff>